<commit_message>
Addendum A: delivery data moved to v4, corrected substitution register
- Retired the v3 load (Corvina SCH-0441 schedules/events, Kelmore BPO-0438-NN sub-POs and deliveries)
- Corvina: builder programme only (SCH-0141-01/02, 49 events, no blanket, no status)
- Kelmore: 26 schedule lines (6 ALT with written basis), 25 per-event sub-POs SPO-0438-01..25 with
  location and source tier (17/4/4), 25 deliveries, 286 call-up lines; event dates and statuses refreshed
- Order.SPAISourceTier added and shown on the Orders Fulfilment tab
- Substitution register: original 99 rules (22 passing the floor) replaced by the corrected 45 (34 passing);
  StaleReason deliberately not loaded
- verify.py: Addendum A6 checks and rule-floor count; order schedule generator reads the v4 programme

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/meridian-data-v2/Corvina_Quarter_BPO-0441_Order_Schedule.xlsx
+++ b/meridian-data-v2/Corvina_Quarter_BPO-0441_Order_Schedule.xlsx
@@ -649,7 +649,7 @@
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>APPLIANCES - delivery schedule SCH-0441-01</t>
+          <t>APPLIANCES - delivery schedule SCH-0141-01</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
     <row r="44">
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>TAPWARE &amp; SANITARYWARE - delivery schedule SCH-0441-02</t>
+          <t>TAPWARE &amp; SANITARYWARE - delivery schedule SCH-0141-02</t>
         </is>
       </c>
     </row>

</xml_diff>